<commit_message>
Add Lavazza FY2020-FY2025 metrics sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wn54G6GwkVyyHQA9rv16MJ
</commit_message>
<xml_diff>
--- a/research/HumanBean_Ziggis_FDD.xlsx
+++ b/research/HumanBean_Ziggis_FDD.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="FDD Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Lavazza" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,9 +17,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="#,##0.0"/>
+    <numFmt numFmtId="167" formatCode="#,##0;(#,##0)"/>
+    <numFmt numFmtId="168" formatCode="0.000"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -79,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -106,6 +110,28 @@
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -261,6 +287,71 @@
     <comment ref="G25" authorId="0" shapeId="0">
       <text>
         <t>Calculated by Claude from the 4 stores listed individually in Item 19</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Claude</author>
+  </authors>
+  <commentList>
+    <comment ref="E6" authorId="0" shapeId="0">
+      <text>
+        <t>Includes 9 months of MaxiCoffee (acquired March 2023)</t>
+      </text>
+    </comment>
+    <comment ref="B15" authorId="0" shapeId="0">
+      <text>
+        <t>As restated in the 2022 report</t>
+      </text>
+    </comment>
+    <comment ref="E15" authorId="0" shapeId="0">
+      <text>
+        <t>Turned negative after the MaxiCoffee acquisition</t>
+      </text>
+    </comment>
+    <comment ref="F15" authorId="0" shapeId="0">
+      <text>
+        <t>49% stake in IVS Group acquired in 2024</t>
+      </text>
+    </comment>
+    <comment ref="E17" authorId="0" shapeId="0">
+      <text>
+        <t>Cash flow from operating activities, as described in the 2023 report</t>
+      </text>
+    </comment>
+    <comment ref="D20" authorId="0" shapeId="0">
+      <text>
+        <t>As reported. The 2023 report restated FY2022 to €1,279.5M after moving the UK into Non-EU</t>
+      </text>
+    </comment>
+    <comment ref="D21" authorId="0" shapeId="0">
+      <text>
+        <t>As reported. Restated to €714.2M in the 2023 report</t>
+      </text>
+    </comment>
+    <comment ref="B27" authorId="0" shapeId="0">
+      <text>
+        <t>Retail channel growth, as stated in the 2020 report</t>
+      </text>
+    </comment>
+    <comment ref="B31" authorId="0" shapeId="0">
+      <text>
+        <t>Stated as 'over 4,000'</t>
+      </text>
+    </comment>
+    <comment ref="E31" authorId="0" shapeId="0">
+      <text>
+        <t>Rise includes MaxiCoffee</t>
+      </text>
+    </comment>
+    <comment ref="G35" authorId="0" shapeId="0">
+      <text>
+        <t>Approximate; check against the ECB annual average</t>
       </text>
     </comment>
   </commentList>
@@ -1295,4 +1386,957 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Lavazza Group: Reported Metrics FY2020–FY2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Source: Lavazza Group consolidated annual reports (IFRS). € millions unless noted. Lavazza does not report US revenue on its own.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>FY2020</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>FY2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Group P&amp;L (consolidated)</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n"/>
+      <c r="C5" s="7" t="n"/>
+      <c r="D5" s="7" t="n"/>
+      <c r="E5" s="7" t="n"/>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="7" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="n">
+        <v>2085.3</v>
+      </c>
+      <c r="C6" s="18" t="n">
+        <v>2308.4</v>
+      </c>
+      <c r="D6" s="18" t="n">
+        <v>2715.5</v>
+      </c>
+      <c r="E6" s="19" t="n">
+        <v>3068.9</v>
+      </c>
+      <c r="F6" s="18" t="n">
+        <v>3349.1</v>
+      </c>
+      <c r="G6" s="18" t="n">
+        <v>3875.3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Revenue growth (YoY)</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="n">
+        <v>-0.052</v>
+      </c>
+      <c r="C7" s="20">
+        <f>C6/B6-1</f>
+        <v/>
+      </c>
+      <c r="D7" s="20">
+        <f>D6/C6-1</f>
+        <v/>
+      </c>
+      <c r="E7" s="20">
+        <f>E6/D6-1</f>
+        <v/>
+      </c>
+      <c r="F7" s="20">
+        <f>F6/E6-1</f>
+        <v/>
+      </c>
+      <c r="G7" s="20">
+        <f>G6/F6-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="n">
+        <v>252.8</v>
+      </c>
+      <c r="C8" s="21" t="n">
+        <v>312</v>
+      </c>
+      <c r="D8" s="21" t="n">
+        <v>309</v>
+      </c>
+      <c r="E8" s="21" t="n">
+        <v>263</v>
+      </c>
+      <c r="F8" s="21" t="n">
+        <v>312.1</v>
+      </c>
+      <c r="G8" s="21" t="n">
+        <v>339.6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>EBITDA margin</t>
+        </is>
+      </c>
+      <c r="B9" s="20">
+        <f>B8/B6</f>
+        <v/>
+      </c>
+      <c r="C9" s="20">
+        <f>C8/C6</f>
+        <v/>
+      </c>
+      <c r="D9" s="20">
+        <f>D8/D6</f>
+        <v/>
+      </c>
+      <c r="E9" s="20">
+        <f>E8/E6</f>
+        <v/>
+      </c>
+      <c r="F9" s="20">
+        <f>F8/F6</f>
+        <v/>
+      </c>
+      <c r="G9" s="20">
+        <f>G8/G6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>EBITDA margin (as reported)</t>
+        </is>
+      </c>
+      <c r="B10" s="20" t="n">
+        <v>0.121</v>
+      </c>
+      <c r="C10" s="20" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="D10" s="20" t="n">
+        <v>0.114</v>
+      </c>
+      <c r="E10" s="20" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+      <c r="F10" s="20" t="n">
+        <v>0.093</v>
+      </c>
+      <c r="G10" s="20" t="n">
+        <v>0.08799999999999999</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>EBIT</t>
+        </is>
+      </c>
+      <c r="B11" s="21" t="n">
+        <v>107.7</v>
+      </c>
+      <c r="C11" s="21" t="n">
+        <v>164</v>
+      </c>
+      <c r="D11" s="21" t="n">
+        <v>160</v>
+      </c>
+      <c r="E11" s="21" t="n">
+        <v>97</v>
+      </c>
+      <c r="F11" s="21" t="n">
+        <v>130.5</v>
+      </c>
+      <c r="G11" s="21" t="n">
+        <v>157.1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>EBIT margin</t>
+        </is>
+      </c>
+      <c r="B12" s="20">
+        <f>B11/B6</f>
+        <v/>
+      </c>
+      <c r="C12" s="20">
+        <f>C11/C6</f>
+        <v/>
+      </c>
+      <c r="D12" s="20">
+        <f>D11/D6</f>
+        <v/>
+      </c>
+      <c r="E12" s="20">
+        <f>E11/E6</f>
+        <v/>
+      </c>
+      <c r="F12" s="20">
+        <f>F11/F6</f>
+        <v/>
+      </c>
+      <c r="G12" s="20">
+        <f>G11/G6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Net profit (Group consolidated result)</t>
+        </is>
+      </c>
+      <c r="B13" s="21" t="n">
+        <v>72.90000000000001</v>
+      </c>
+      <c r="C13" s="21" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="D13" s="21" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="E13" s="21" t="n">
+        <v>67.90000000000001</v>
+      </c>
+      <c r="F13" s="21" t="n">
+        <v>82.40000000000001</v>
+      </c>
+      <c r="G13" s="21" t="n">
+        <v>91.7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Balance sheet / cash</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="7" t="n"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="7" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Net financial position (+ cash / − debt)</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="n">
+        <v>102</v>
+      </c>
+      <c r="C15" s="23" t="n">
+        <v>283</v>
+      </c>
+      <c r="D15" s="23" t="n">
+        <v>136</v>
+      </c>
+      <c r="E15" s="22" t="n">
+        <v>-292</v>
+      </c>
+      <c r="F15" s="22" t="n">
+        <v>-511</v>
+      </c>
+      <c r="G15" s="23" t="n">
+        <v>-432</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Free cash flow</t>
+        </is>
+      </c>
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="C16" s="24" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="D16" s="24" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E16" s="24" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F16" s="24" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G16" s="21" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Operating cash generation</t>
+        </is>
+      </c>
+      <c r="B17" s="25" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="n">
+        <v>203</v>
+      </c>
+      <c r="D17" s="25" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E17" s="22" t="n">
+        <v>-17</v>
+      </c>
+      <c r="F17" s="25" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G17" s="25" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Revenue by geography (IFRS 15 note)</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="7" t="n"/>
+      <c r="D18" s="7" t="n"/>
+      <c r="E18" s="7" t="n"/>
+      <c r="F18" s="7" t="n"/>
+      <c r="G18" s="7" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="B19" s="21" t="n">
+        <v>630.2</v>
+      </c>
+      <c r="C19" s="21" t="n">
+        <v>671.2</v>
+      </c>
+      <c r="D19" s="21" t="n">
+        <v>721.7</v>
+      </c>
+      <c r="E19" s="21" t="n">
+        <v>754.5</v>
+      </c>
+      <c r="F19" s="21" t="n">
+        <v>782.2</v>
+      </c>
+      <c r="G19" s="21" t="n">
+        <v>901.3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Other EU countries (+ UK through 2022)</t>
+        </is>
+      </c>
+      <c r="B20" s="21" t="n">
+        <v>1046.1</v>
+      </c>
+      <c r="C20" s="21" t="n">
+        <v>1190.3</v>
+      </c>
+      <c r="D20" s="19" t="n">
+        <v>1444.4</v>
+      </c>
+      <c r="E20" s="21" t="n">
+        <v>1562.4</v>
+      </c>
+      <c r="F20" s="21" t="n">
+        <v>1725.3</v>
+      </c>
+      <c r="G20" s="21" t="n">
+        <v>1989.1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Non-EU countries (includes North America)</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="n">
+        <v>409</v>
+      </c>
+      <c r="C21" s="18" t="n">
+        <v>447</v>
+      </c>
+      <c r="D21" s="19" t="n">
+        <v>549.3</v>
+      </c>
+      <c r="E21" s="18" t="n">
+        <v>752</v>
+      </c>
+      <c r="F21" s="18" t="n">
+        <v>841.6</v>
+      </c>
+      <c r="G21" s="18" t="n">
+        <v>984.9</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Non-EU share of revenue</t>
+        </is>
+      </c>
+      <c r="B22" s="20">
+        <f>B21/B6</f>
+        <v/>
+      </c>
+      <c r="C22" s="20">
+        <f>C21/C6</f>
+        <v/>
+      </c>
+      <c r="D22" s="20">
+        <f>D21/D6</f>
+        <v/>
+      </c>
+      <c r="E22" s="20">
+        <f>E21/E6</f>
+        <v/>
+      </c>
+      <c r="F22" s="20">
+        <f>F21/F6</f>
+        <v/>
+      </c>
+      <c r="G22" s="20">
+        <f>G21/G6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>US / North America disclosures (growth rates only; no dollar amounts)</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="n"/>
+      <c r="C23" s="7" t="n"/>
+      <c r="D23" s="7" t="n"/>
+      <c r="E23" s="7" t="n"/>
+      <c r="F23" s="7" t="n"/>
+      <c r="G23" s="7" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>North America revenue growth</t>
+        </is>
+      </c>
+      <c r="B24" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="C24" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="D24" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E24" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F24" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G24" s="20" t="n">
+        <v>0.269</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>US sales growth</t>
+        </is>
+      </c>
+      <c r="B25" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="C25" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="D25" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E25" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F25" s="20" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="G25" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>North America retail-channel revenue growth</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="C26" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="D26" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E26" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F26" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G26" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>US retail sell-out growth (by value)</t>
+        </is>
+      </c>
+      <c r="B27" s="27" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="C27" s="20" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="D27" s="20" t="n">
+        <v>0.141</v>
+      </c>
+      <c r="E27" s="20" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="F27" s="20" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="G27" s="20" t="n">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Canada retail-channel growth</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="n">
+        <v>0.285</v>
+      </c>
+      <c r="C28" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="D28" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E28" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F28" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G28" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>North America volume growth</t>
+        </is>
+      </c>
+      <c r="B29" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="C29" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="D29" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="E29" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="F29" s="26" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G29" s="20" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="n"/>
+      <c r="C30" s="7" t="n"/>
+      <c r="D30" s="7" t="n"/>
+      <c r="E30" s="7" t="n"/>
+      <c r="F30" s="7" t="n"/>
+      <c r="G30" s="7" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Group employees (approx., as stated)</t>
+        </is>
+      </c>
+      <c r="B31" s="28" t="n">
+        <v>4000</v>
+      </c>
+      <c r="C31" s="13" t="n">
+        <v>4200</v>
+      </c>
+      <c r="D31" s="13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E31" s="28" t="n">
+        <v>5500</v>
+      </c>
+      <c r="F31" s="29" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G31" s="13" t="n">
+        <v>5800</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Parent company headcount (Luigi Lavazza S.p.A.)</t>
+        </is>
+      </c>
+      <c r="B32" s="13" t="n">
+        <v>1741</v>
+      </c>
+      <c r="C32" s="13" t="n">
+        <v>1781</v>
+      </c>
+      <c r="D32" s="13" t="n">
+        <v>1790</v>
+      </c>
+      <c r="E32" s="13" t="n">
+        <v>1854</v>
+      </c>
+      <c r="F32" s="13" t="n">
+        <v>1843</v>
+      </c>
+      <c r="G32" s="29" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Parent company capex</t>
+        </is>
+      </c>
+      <c r="B33" s="21" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="C33" s="21" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="D33" s="21" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="E33" s="21" t="n">
+        <v>50.1</v>
+      </c>
+      <c r="F33" s="24" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G33" s="24" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>FX helper (approximate ECB annual average EUR/USD)</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="n"/>
+      <c r="C34" s="7" t="n"/>
+      <c r="D34" s="7" t="n"/>
+      <c r="E34" s="7" t="n"/>
+      <c r="F34" s="7" t="n"/>
+      <c r="G34" s="7" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="B35" s="30" t="n">
+        <v>1.142</v>
+      </c>
+      <c r="C35" s="30" t="n">
+        <v>1.183</v>
+      </c>
+      <c r="D35" s="30" t="n">
+        <v>1.053</v>
+      </c>
+      <c r="E35" s="30" t="n">
+        <v>1.081</v>
+      </c>
+      <c r="F35" s="30" t="n">
+        <v>1.082</v>
+      </c>
+      <c r="G35" s="31" t="n">
+        <v>1.13</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Revenue in US$ millions</t>
+        </is>
+      </c>
+      <c r="B36" s="13">
+        <f>B6*B35</f>
+        <v/>
+      </c>
+      <c r="C36" s="13">
+        <f>C6*C35</f>
+        <v/>
+      </c>
+      <c r="D36" s="13">
+        <f>D6*D35</f>
+        <v/>
+      </c>
+      <c r="E36" s="13">
+        <f>E6*E35</f>
+        <v/>
+      </c>
+      <c r="F36" s="13">
+        <f>F6*F35</f>
+        <v/>
+      </c>
+      <c r="G36" s="13">
+        <f>G6*G35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Non-EU revenue in US$ millions</t>
+        </is>
+      </c>
+      <c r="B37" s="13">
+        <f>B21*B35</f>
+        <v/>
+      </c>
+      <c r="C37" s="13">
+        <f>C21*C35</f>
+        <v/>
+      </c>
+      <c r="D37" s="13">
+        <f>D21*D35</f>
+        <v/>
+      </c>
+      <c r="E37" s="13">
+        <f>E21*E35</f>
+        <v/>
+      </c>
+      <c r="F37" s="13">
+        <f>F21*F35</f>
+        <v/>
+      </c>
+      <c r="G37" s="13">
+        <f>G21*G35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Orange = not disclosed that year. Grey italic = see cell comment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Reports: lavazzagroup.com/en/who-we-are/results.html (FY2020–FY2025 annual reports)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
 </file>
</xml_diff>